<commit_message>
Update dTimes.xlsx from colleague's branch and regenerate data
https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/dTimes.xlsx
+++ b/dTimes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/Área de Trabalho/dash-ticket/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="8_{5B5F332C-664E-451E-A267-741B67AA2ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A7992B2-BCC5-452A-B6E2-F40836C321CE}"/>
+  <xr:revisionPtr revIDLastSave="178" documentId="8_{5B5F332C-664E-451E-A267-741B67AA2ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCA265E2-EF1C-4A62-82D8-04E2684CC4CE}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C78CE2AA-518B-4E7B-ADE2-2214072EC913}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="355">
   <si>
     <t>Flamengo</t>
   </si>
@@ -1079,9 +1079,6 @@
     <t>121JUBRCS</t>
   </si>
   <si>
-    <t>IMAGENS</t>
-  </si>
-  <si>
     <t>Capital</t>
   </si>
   <si>
@@ -1094,9 +1091,6 @@
     <t>122CABRDF</t>
   </si>
   <si>
-    <t>https://upload.wikimedia.org/wikipedia/commons/thumb/9/96/Clube_de_Regatas_do_Flamengo_logo.svg/960px-Clube_de_Regatas_do_Flamengo_logo.svg.png</t>
-  </si>
-  <si>
     <t>Nacional de Potosí</t>
   </si>
   <si>
@@ -1107,13 +1101,16 @@
   </si>
   <si>
     <t>123NABOPO</t>
+  </si>
+  <si>
+    <t>Pontuação</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1125,14 +1122,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1155,17 +1144,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1504,7 +1491,7 @@
     <col min="1" max="1" width="11.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="131.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -1524,7 +1511,7 @@
         <v>344</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -1543,8 +1530,8 @@
       <c r="E2" t="s">
         <v>136</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>351</v>
+      <c r="F2" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -1563,7 +1550,9 @@
       <c r="E3" t="s">
         <v>136</v>
       </c>
-      <c r="F3" s="2"/>
+      <c r="F3" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -1581,7 +1570,9 @@
       <c r="E4" t="s">
         <v>136</v>
       </c>
-      <c r="F4" s="2"/>
+      <c r="F4" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -1599,7 +1590,9 @@
       <c r="E5" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="2"/>
+      <c r="F5" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -1617,7 +1610,9 @@
       <c r="E6" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="2"/>
+      <c r="F6" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1635,6 +1630,9 @@
       <c r="E7" t="s">
         <v>5</v>
       </c>
+      <c r="F7" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -1652,7 +1650,9 @@
       <c r="E8" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="2"/>
+      <c r="F8" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -1670,7 +1670,9 @@
       <c r="E9" t="s">
         <v>143</v>
       </c>
-      <c r="F9" s="2"/>
+      <c r="F9" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -1688,7 +1690,9 @@
       <c r="E10" t="s">
         <v>144</v>
       </c>
-      <c r="F10" s="2"/>
+      <c r="F10" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
@@ -1706,7 +1710,9 @@
       <c r="E11" t="s">
         <v>144</v>
       </c>
-      <c r="F11" s="2"/>
+      <c r="F11" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -1724,6 +1730,9 @@
       <c r="E12" t="s">
         <v>145</v>
       </c>
+      <c r="F12" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -1741,6 +1750,9 @@
       <c r="E13" t="s">
         <v>146</v>
       </c>
+      <c r="F13" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
@@ -1758,7 +1770,9 @@
       <c r="E14" t="s">
         <v>145</v>
       </c>
-      <c r="F14" s="2"/>
+      <c r="F14" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
@@ -1776,7 +1790,9 @@
       <c r="E15" t="s">
         <v>147</v>
       </c>
-      <c r="F15" s="2"/>
+      <c r="F15" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -1794,7 +1810,9 @@
       <c r="E16" t="s">
         <v>147</v>
       </c>
-      <c r="F16" s="2"/>
+      <c r="F16" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
@@ -1812,7 +1830,9 @@
       <c r="E17" t="s">
         <v>148</v>
       </c>
-      <c r="F17" s="2"/>
+      <c r="F17" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
@@ -1830,6 +1850,9 @@
       <c r="E18" t="s">
         <v>148</v>
       </c>
+      <c r="F18" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
@@ -1847,6 +1870,9 @@
       <c r="E19" t="s">
         <v>147</v>
       </c>
+      <c r="F19" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
@@ -1864,7 +1890,9 @@
       <c r="E20" t="s">
         <v>149</v>
       </c>
-      <c r="F20" s="2"/>
+      <c r="F20" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
@@ -1882,7 +1910,9 @@
       <c r="E21" t="s">
         <v>19</v>
       </c>
-      <c r="F21" s="2"/>
+      <c r="F21" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
@@ -1900,7 +1930,9 @@
       <c r="E22" t="s">
         <v>149</v>
       </c>
-      <c r="F22" s="2"/>
+      <c r="F22" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
@@ -1918,6 +1950,9 @@
       <c r="E23" t="s">
         <v>19</v>
       </c>
+      <c r="F23" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
@@ -1935,7 +1970,9 @@
       <c r="E24" t="s">
         <v>22</v>
       </c>
-      <c r="F24" s="2"/>
+      <c r="F24" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
@@ -1953,7 +1990,9 @@
       <c r="E25" t="s">
         <v>23</v>
       </c>
-      <c r="F25" s="2"/>
+      <c r="F25" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
@@ -1971,6 +2010,9 @@
       <c r="E26" t="s">
         <v>24</v>
       </c>
+      <c r="F26" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
@@ -1988,6 +2030,9 @@
       <c r="E27" t="s">
         <v>140</v>
       </c>
+      <c r="F27" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
@@ -2005,6 +2050,9 @@
       <c r="E28" t="s">
         <v>141</v>
       </c>
+      <c r="F28" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
@@ -2022,6 +2070,9 @@
       <c r="E29" t="s">
         <v>142</v>
       </c>
+      <c r="F29" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
@@ -2039,6 +2090,9 @@
       <c r="E30" t="s">
         <v>150</v>
       </c>
+      <c r="F30" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
@@ -2056,6 +2110,9 @@
       <c r="E31" t="s">
         <v>151</v>
       </c>
+      <c r="F31" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
@@ -2073,8 +2130,11 @@
       <c r="E32" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F32" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>251</v>
       </c>
@@ -2090,8 +2150,11 @@
       <c r="E33" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F33" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>252</v>
       </c>
@@ -2107,8 +2170,11 @@
       <c r="E34" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F34" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>253</v>
       </c>
@@ -2124,8 +2190,11 @@
       <c r="E35" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F35" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>254</v>
       </c>
@@ -2141,8 +2210,11 @@
       <c r="E36" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F36" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>255</v>
       </c>
@@ -2158,8 +2230,11 @@
       <c r="E37" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F37" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>256</v>
       </c>
@@ -2175,8 +2250,11 @@
       <c r="E38" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F38" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>257</v>
       </c>
@@ -2192,8 +2270,11 @@
       <c r="E39" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F39" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>258</v>
       </c>
@@ -2209,8 +2290,11 @@
       <c r="E40" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F40" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>259</v>
       </c>
@@ -2226,8 +2310,11 @@
       <c r="E41" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F41" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>260</v>
       </c>
@@ -2243,8 +2330,11 @@
       <c r="E42" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F42" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>261</v>
       </c>
@@ -2260,8 +2350,11 @@
       <c r="E43" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F43" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>262</v>
       </c>
@@ -2277,8 +2370,11 @@
       <c r="E44" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F44" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>263</v>
       </c>
@@ -2294,8 +2390,11 @@
       <c r="E45" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F45" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>264</v>
       </c>
@@ -2311,8 +2410,11 @@
       <c r="E46" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F46" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>265</v>
       </c>
@@ -2328,8 +2430,11 @@
       <c r="E47" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F47" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>266</v>
       </c>
@@ -2345,8 +2450,11 @@
       <c r="E48" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F48" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>267</v>
       </c>
@@ -2362,8 +2470,11 @@
       <c r="E49" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F49" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>268</v>
       </c>
@@ -2379,8 +2490,11 @@
       <c r="E50" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F50" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>269</v>
       </c>
@@ -2396,8 +2510,11 @@
       <c r="E51" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F51" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>270</v>
       </c>
@@ -2413,8 +2530,11 @@
       <c r="E52" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F52" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>271</v>
       </c>
@@ -2430,8 +2550,11 @@
       <c r="E53" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F53" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>272</v>
       </c>
@@ -2447,8 +2570,11 @@
       <c r="E54" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F54" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>273</v>
       </c>
@@ -2464,8 +2590,11 @@
       <c r="E55" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F55" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>274</v>
       </c>
@@ -2481,8 +2610,11 @@
       <c r="E56" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F56" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>275</v>
       </c>
@@ -2498,8 +2630,11 @@
       <c r="E57" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F57" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>276</v>
       </c>
@@ -2515,8 +2650,11 @@
       <c r="E58" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F58" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>277</v>
       </c>
@@ -2532,8 +2670,11 @@
       <c r="E59" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F59" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>278</v>
       </c>
@@ -2549,8 +2690,11 @@
       <c r="E60" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F60" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>279</v>
       </c>
@@ -2566,8 +2710,11 @@
       <c r="E61" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F61" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>280</v>
       </c>
@@ -2583,8 +2730,11 @@
       <c r="E62" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F62" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>281</v>
       </c>
@@ -2600,8 +2750,11 @@
       <c r="E63" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F63" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>282</v>
       </c>
@@ -2617,8 +2770,11 @@
       <c r="E64" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F64" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>283</v>
       </c>
@@ -2634,8 +2790,11 @@
       <c r="E65" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F65" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>284</v>
       </c>
@@ -2651,8 +2810,11 @@
       <c r="E66" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F66" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>285</v>
       </c>
@@ -2668,8 +2830,11 @@
       <c r="E67" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F67" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>286</v>
       </c>
@@ -2685,8 +2850,11 @@
       <c r="E68" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F68" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>287</v>
       </c>
@@ -2702,8 +2870,11 @@
       <c r="E69" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F69" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>288</v>
       </c>
@@ -2719,8 +2890,11 @@
       <c r="E70" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F70" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>289</v>
       </c>
@@ -2736,8 +2910,11 @@
       <c r="E71" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F71" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>290</v>
       </c>
@@ -2753,8 +2930,11 @@
       <c r="E72" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F72" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>291</v>
       </c>
@@ -2770,8 +2950,11 @@
       <c r="E73" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F73" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>292</v>
       </c>
@@ -2787,8 +2970,11 @@
       <c r="E74" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F74" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>293</v>
       </c>
@@ -2804,8 +2990,11 @@
       <c r="E75" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F75" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>294</v>
       </c>
@@ -2821,8 +3010,11 @@
       <c r="E76" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F76" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>295</v>
       </c>
@@ -2838,8 +3030,11 @@
       <c r="E77" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F77" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>296</v>
       </c>
@@ -2855,8 +3050,11 @@
       <c r="E78" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F78" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>297</v>
       </c>
@@ -2872,8 +3070,11 @@
       <c r="E79" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F79" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>298</v>
       </c>
@@ -2889,8 +3090,11 @@
       <c r="E80" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F80" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>299</v>
       </c>
@@ -2906,8 +3110,11 @@
       <c r="E81" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F81" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>300</v>
       </c>
@@ -2923,8 +3130,11 @@
       <c r="E82" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F82" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>301</v>
       </c>
@@ -2940,8 +3150,11 @@
       <c r="E83" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F83" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>302</v>
       </c>
@@ -2957,8 +3170,11 @@
       <c r="E84" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F84" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>303</v>
       </c>
@@ -2974,8 +3190,11 @@
       <c r="E85" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F85" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>304</v>
       </c>
@@ -2991,8 +3210,11 @@
       <c r="E86" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F86" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>305</v>
       </c>
@@ -3008,8 +3230,11 @@
       <c r="E87" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F87" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>306</v>
       </c>
@@ -3025,8 +3250,11 @@
       <c r="E88" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F88" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>307</v>
       </c>
@@ -3042,8 +3270,11 @@
       <c r="E89" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F89" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>308</v>
       </c>
@@ -3059,8 +3290,11 @@
       <c r="E90" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F90" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>220</v>
       </c>
@@ -3076,8 +3310,11 @@
       <c r="E91" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F91" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>309</v>
       </c>
@@ -3093,8 +3330,11 @@
       <c r="E92" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F92" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>310</v>
       </c>
@@ -3110,8 +3350,11 @@
       <c r="E93" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F93" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>311</v>
       </c>
@@ -3127,8 +3370,11 @@
       <c r="E94" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F94" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>312</v>
       </c>
@@ -3144,8 +3390,11 @@
       <c r="E95" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F95" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>313</v>
       </c>
@@ -3161,8 +3410,11 @@
       <c r="E96" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F96" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>314</v>
       </c>
@@ -3178,8 +3430,11 @@
       <c r="E97" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F97" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>315</v>
       </c>
@@ -3195,8 +3450,11 @@
       <c r="E98" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F98" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>316</v>
       </c>
@@ -3212,8 +3470,11 @@
       <c r="E99" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F99" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>317</v>
       </c>
@@ -3229,8 +3490,11 @@
       <c r="E100" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F100" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>318</v>
       </c>
@@ -3246,8 +3510,11 @@
       <c r="E101" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F101" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>319</v>
       </c>
@@ -3263,8 +3530,11 @@
       <c r="E102" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F102" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>320</v>
       </c>
@@ -3280,8 +3550,11 @@
       <c r="E103" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F103" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>321</v>
       </c>
@@ -3297,8 +3570,11 @@
       <c r="E104" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F104" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>322</v>
       </c>
@@ -3314,8 +3590,11 @@
       <c r="E105" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F105" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>323</v>
       </c>
@@ -3331,8 +3610,11 @@
       <c r="E106" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F106" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>324</v>
       </c>
@@ -3348,8 +3630,11 @@
       <c r="E107" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F107" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>325</v>
       </c>
@@ -3365,8 +3650,11 @@
       <c r="E108" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F108" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>326</v>
       </c>
@@ -3382,8 +3670,11 @@
       <c r="E109" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F109" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>327</v>
       </c>
@@ -3399,8 +3690,11 @@
       <c r="E110" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F110" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>328</v>
       </c>
@@ -3416,8 +3710,11 @@
       <c r="E111" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F111" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>329</v>
       </c>
@@ -3432,6 +3729,9 @@
       </c>
       <c r="E112" t="s">
         <v>187</v>
+      </c>
+      <c r="F112" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.35">
@@ -3450,6 +3750,9 @@
       <c r="E113" t="s">
         <v>185</v>
       </c>
+      <c r="F113" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
@@ -3467,6 +3770,9 @@
       <c r="E114" t="s">
         <v>188</v>
       </c>
+      <c r="F114" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
@@ -3484,6 +3790,9 @@
       <c r="E115" t="s">
         <v>97</v>
       </c>
+      <c r="F115" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
@@ -3501,6 +3810,9 @@
       <c r="E116" t="s">
         <v>189</v>
       </c>
+      <c r="F116" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
@@ -3518,6 +3830,9 @@
       <c r="E117" t="s">
         <v>190</v>
       </c>
+      <c r="F117" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
@@ -3535,6 +3850,9 @@
       <c r="E118" t="s">
         <v>192</v>
       </c>
+      <c r="F118" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
@@ -3552,6 +3870,9 @@
       <c r="E119" t="s">
         <v>194</v>
       </c>
+      <c r="F119" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
@@ -3569,6 +3890,9 @@
       <c r="E120" t="s">
         <v>196</v>
       </c>
+      <c r="F120" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
@@ -3586,47 +3910,52 @@
       <c r="E121" t="s">
         <v>340</v>
       </c>
-      <c r="F121" s="2"/>
+      <c r="F121" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B122" t="s">
+        <v>346</v>
+      </c>
+      <c r="C122" t="s">
+        <v>110</v>
+      </c>
+      <c r="D122" t="s">
         <v>347</v>
       </c>
-      <c r="C122" t="s">
-        <v>110</v>
-      </c>
-      <c r="D122" t="s">
+      <c r="E122" t="s">
         <v>348</v>
       </c>
-      <c r="E122" t="s">
-        <v>349</v>
+      <c r="F122" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B123" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C123" t="s">
         <v>103</v>
       </c>
       <c r="D123" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="E123" t="s">
-        <v>353</v>
+        <v>351</v>
+      </c>
+      <c r="F123" s="2">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F123" xr:uid="{DE7E04D1-2798-4098-907E-D4A20ADC6AF9}"/>
-  <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{CD126DD6-0BB8-4D62-BEF2-FB43B4EE069F}"/>
-  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>